<commit_message>
Add test case for owner change
</commit_message>
<xml_diff>
--- a/tests/data/test_data_import/DVV_original.xlsx
+++ b/tests/data/test_data_import/DVV_original.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="3"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="R1 rakennus" sheetId="1" state="visible" r:id="rId2"/>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="242" uniqueCount="150">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="260" uniqueCount="154">
   <si>
     <t xml:space="preserve">Rakennustunnus</t>
   </si>
@@ -170,6 +170,12 @@
     <t xml:space="preserve">398</t>
   </si>
   <si>
+    <t xml:space="preserve">200000001A</t>
+  </si>
+  <si>
+    <t xml:space="preserve">39800200020001</t>
+  </si>
+  <si>
     <t xml:space="preserve">Osoite-numero</t>
   </si>
   <si>
@@ -355,6 +361,12 @@
   </si>
   <si>
     <t xml:space="preserve">Granström Otto</t>
+  </si>
+  <si>
+    <t xml:space="preserve">220752-848C</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pohjonen Aarno Armas</t>
   </si>
   <si>
     <t xml:space="preserve">Huo-neisto-kirjain</t>
@@ -724,7 +736,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:Z6"/>
+  <dimension ref="A1:Z7"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="11.53"/>
@@ -1132,6 +1144,68 @@
         <v>6765134</v>
       </c>
       <c r="Y6" s="2" t="n">
+        <v>428759</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="C7" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="D7" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="F7" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="G7" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="H7" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J7" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="K7" s="2" t="n">
+        <v>19750101</v>
+      </c>
+      <c r="L7" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="N7" s="2" t="n">
+        <v>80</v>
+      </c>
+      <c r="O7" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q7" s="2" t="n">
+        <v>250</v>
+      </c>
+      <c r="S7" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="T7" s="2" t="n">
+        <v>19780101</v>
+      </c>
+      <c r="U7" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="V7" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="W7" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="X7" s="2" t="n">
+        <v>6765234</v>
+      </c>
+      <c r="Y7" s="2" t="n">
         <v>428759</v>
       </c>
     </row>
@@ -1151,7 +1225,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:I6"/>
+  <dimension ref="A1:I7"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="11.53"/>
@@ -1167,25 +1241,25 @@
         <v>1</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="D1" s="6" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="E1" s="6" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="F1" s="10" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="G1" s="4" t="s">
         <v>9</v>
       </c>
       <c r="H1" s="6" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="I1" s="6" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1199,10 +1273,10 @@
         <v>1</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="F2" s="2" t="n">
         <v>1</v>
@@ -1211,10 +1285,10 @@
         <v>29</v>
       </c>
       <c r="H2" s="2" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="I2" s="2" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1228,7 +1302,7 @@
         <v>1</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="E3" s="2"/>
       <c r="F3" s="2" t="n">
@@ -1238,10 +1312,10 @@
         <v>35</v>
       </c>
       <c r="H3" s="2" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="I3" s="2" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1255,7 +1329,7 @@
         <v>1</v>
       </c>
       <c r="D4" s="9" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="F4" s="9" t="n">
         <v>44</v>
@@ -1264,10 +1338,10 @@
         <v>15100</v>
       </c>
       <c r="H4" s="9" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="I4" s="9" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1281,19 +1355,19 @@
         <v>1</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="F5" s="1" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="G5" s="1" t="s">
         <v>43</v>
       </c>
       <c r="H5" s="2" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="I5" s="2" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1307,7 +1381,7 @@
         <v>1</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="F6" s="2" t="n">
         <v>9</v>
@@ -1316,10 +1390,36 @@
         <v>35</v>
       </c>
       <c r="H6" s="2" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="I6" s="2" t="s">
-        <v>60</v>
+        <v>62</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="9" t="s">
+        <v>48</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="C7" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="F7" s="2" t="n">
+        <v>11</v>
+      </c>
+      <c r="G7" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="H7" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="I7" s="2" t="s">
+        <v>62</v>
       </c>
     </row>
   </sheetData>
@@ -1338,7 +1438,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:X6"/>
+  <dimension ref="A1:X7"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="2" width="34.35"/>
@@ -1354,70 +1454,70 @@
         <v>1</v>
       </c>
       <c r="C1" s="10" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="D1" s="11" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="E1" s="5" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="F1" s="5" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="G1" s="5" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="H1" s="4" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="I1" s="12" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="J1" s="4" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="K1" s="13" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="L1" s="5" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="M1" s="6" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="N1" s="4" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="O1" s="6" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="P1" s="5" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="Q1" s="6" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="R1" s="4" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="S1" s="14" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="T1" s="14" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="U1" s="14" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="V1" s="14" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="W1" s="4" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="X1" s="14" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1428,7 +1528,7 @@
         <v>27</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="D2" s="9"/>
       <c r="F2" s="9" t="n">
@@ -1438,37 +1538,37 @@
         <v>1</v>
       </c>
       <c r="H2" s="8" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="I2" s="9" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="J2" s="2" t="n">
         <v>444</v>
       </c>
       <c r="K2" s="2" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="M2" s="2" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="N2" s="8" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="O2" s="2" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="P2" s="2" t="n">
         <v>20100101</v>
       </c>
       <c r="Q2" s="9" t="s">
+        <v>97</v>
+      </c>
+      <c r="R2" s="1" t="s">
         <v>95</v>
       </c>
-      <c r="R2" s="1" t="s">
-        <v>93</v>
-      </c>
       <c r="S2" s="9" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1479,7 +1579,7 @@
         <v>27</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="D3" s="9"/>
       <c r="F3" s="9" t="n">
@@ -1489,25 +1589,25 @@
         <v>1</v>
       </c>
       <c r="H3" s="8" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="I3" s="9" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="J3" s="1" t="s">
         <v>27</v>
       </c>
       <c r="K3" s="2" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="M3" s="2" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="N3" s="8" t="s">
         <v>35</v>
       </c>
       <c r="O3" s="2" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="P3" s="2" t="n">
         <v>20220101</v>
@@ -1523,7 +1623,7 @@
         <v>398</v>
       </c>
       <c r="D4" s="9" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="F4" s="9" t="n">
         <v>20100101</v>
@@ -1535,16 +1635,16 @@
         <v>30</v>
       </c>
       <c r="I4" s="9" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="Q4" s="9" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="R4" s="1" t="n">
         <v>15100</v>
       </c>
       <c r="S4" s="9" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1555,7 +1655,7 @@
         <v>560</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="F5" s="2" t="n">
         <v>19980601</v>
@@ -1564,25 +1664,25 @@
         <v>1</v>
       </c>
       <c r="H5" s="8" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="I5" s="2" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="J5" s="1" t="s">
         <v>41</v>
       </c>
       <c r="K5" s="2" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="M5" s="2" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="N5" s="1" t="n">
         <v>16200</v>
       </c>
       <c r="O5" s="2" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="P5" s="2" t="n">
         <v>19860101</v>
@@ -1596,7 +1696,7 @@
         <v>398</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="F6" s="2" t="n">
         <v>20010601</v>
@@ -1605,16 +1705,45 @@
         <v>1</v>
       </c>
       <c r="H6" s="8" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="I6" s="2" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="J6" s="2" t="n">
         <v>398</v>
       </c>
       <c r="K6" s="2" t="s">
-        <v>99</v>
+        <v>101</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="9" t="s">
+        <v>48</v>
+      </c>
+      <c r="B7" s="1" t="n">
+        <v>398</v>
+      </c>
+      <c r="C7" s="0" t="s">
+        <v>112</v>
+      </c>
+      <c r="F7" s="2" t="n">
+        <v>20010601</v>
+      </c>
+      <c r="G7" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="H7" s="8" t="s">
+        <v>91</v>
+      </c>
+      <c r="I7" s="2" t="s">
+        <v>113</v>
+      </c>
+      <c r="J7" s="2" t="n">
+        <v>398</v>
+      </c>
+      <c r="K7" s="2" t="s">
+        <v>101</v>
       </c>
     </row>
   </sheetData>
@@ -1650,43 +1779,43 @@
         <v>1</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>110</v>
+        <v>114</v>
       </c>
       <c r="D1" s="4" t="s">
-        <v>111</v>
+        <v>115</v>
       </c>
       <c r="E1" s="5" t="s">
-        <v>112</v>
+        <v>116</v>
       </c>
       <c r="F1" s="5" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="G1" s="15" t="s">
-        <v>113</v>
+        <v>117</v>
       </c>
       <c r="H1" s="16" t="s">
-        <v>114</v>
+        <v>118</v>
       </c>
       <c r="I1" s="16" t="s">
-        <v>115</v>
+        <v>119</v>
       </c>
       <c r="J1" s="6" t="s">
-        <v>116</v>
+        <v>120</v>
       </c>
       <c r="K1" s="4" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="L1" s="6" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="M1" s="5" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="N1" s="17" t="s">
-        <v>117</v>
+        <v>121</v>
       </c>
       <c r="O1" s="17" t="s">
-        <v>118</v>
+        <v>122</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1697,34 +1826,34 @@
         <v>27</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>119</v>
+        <v>123</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>120</v>
+        <v>124</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>119</v>
+        <v>123</v>
       </c>
       <c r="F2" s="2" t="n">
         <v>1</v>
       </c>
       <c r="G2" s="9" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="H2" s="9" t="s">
-        <v>121</v>
+        <v>125</v>
       </c>
       <c r="I2" s="9" t="s">
-        <v>122</v>
+        <v>126</v>
       </c>
       <c r="J2" s="2" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="K2" s="8" t="n">
         <v>15230</v>
       </c>
       <c r="L2" s="2" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="M2" s="2" t="n">
         <v>20220101</v>
@@ -1747,31 +1876,31 @@
         <v>45</v>
       </c>
       <c r="D3" s="1" t="s">
+        <v>127</v>
+      </c>
+      <c r="E3" s="2" t="s">
         <v>123</v>
       </c>
-      <c r="E3" s="2" t="s">
-        <v>119</v>
-      </c>
       <c r="F3" s="9" t="n">
         <v>1</v>
       </c>
       <c r="G3" s="9" t="s">
-        <v>124</v>
+        <v>128</v>
       </c>
       <c r="H3" s="9" t="s">
-        <v>125</v>
+        <v>129</v>
       </c>
       <c r="I3" s="9" t="s">
-        <v>126</v>
+        <v>130</v>
       </c>
       <c r="J3" s="9" t="s">
-        <v>127</v>
+        <v>131</v>
       </c>
       <c r="K3" s="1" t="n">
         <v>15100</v>
       </c>
       <c r="L3" s="9" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="M3" s="9" t="n">
         <v>20200101</v>
@@ -1794,31 +1923,31 @@
         <v>45</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>128</v>
+        <v>132</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>119</v>
+        <v>123</v>
       </c>
       <c r="F4" s="9" t="n">
         <v>1</v>
       </c>
       <c r="G4" s="9" t="s">
-        <v>129</v>
+        <v>133</v>
       </c>
       <c r="H4" s="9" t="s">
-        <v>130</v>
+        <v>134</v>
       </c>
       <c r="I4" s="9" t="s">
-        <v>131</v>
+        <v>135</v>
       </c>
       <c r="J4" s="9" t="s">
-        <v>132</v>
+        <v>136</v>
       </c>
       <c r="K4" s="1" t="n">
         <v>15100</v>
       </c>
       <c r="L4" s="9" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="M4" s="9" t="n">
         <v>20210101</v>
@@ -1838,34 +1967,34 @@
         <v>398</v>
       </c>
       <c r="C5" s="9" t="s">
-        <v>133</v>
+        <v>137</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>134</v>
+        <v>138</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>119</v>
+        <v>123</v>
       </c>
       <c r="F5" s="9" t="n">
         <v>1</v>
       </c>
       <c r="G5" s="9" t="s">
-        <v>135</v>
+        <v>139</v>
       </c>
       <c r="H5" s="9" t="s">
-        <v>136</v>
+        <v>140</v>
       </c>
       <c r="I5" s="9" t="s">
-        <v>137</v>
+        <v>141</v>
       </c>
       <c r="J5" s="9" t="s">
-        <v>138</v>
+        <v>142</v>
       </c>
       <c r="K5" s="1" t="n">
         <v>15100</v>
       </c>
       <c r="L5" s="9" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="M5" s="9" t="n">
         <v>20220101</v>
@@ -1885,34 +2014,34 @@
         <v>398</v>
       </c>
       <c r="C6" s="9" t="s">
-        <v>133</v>
+        <v>137</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>139</v>
+        <v>143</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>119</v>
+        <v>123</v>
       </c>
       <c r="F6" s="9" t="n">
         <v>1</v>
       </c>
       <c r="G6" s="9" t="s">
-        <v>140</v>
+        <v>144</v>
       </c>
       <c r="H6" s="9" t="s">
-        <v>141</v>
+        <v>145</v>
       </c>
       <c r="I6" s="9" t="s">
-        <v>142</v>
+        <v>146</v>
       </c>
       <c r="J6" s="9" t="s">
-        <v>143</v>
+        <v>147</v>
       </c>
       <c r="K6" s="1" t="n">
         <v>15100</v>
       </c>
       <c r="L6" s="9" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="M6" s="9" t="n">
         <v>20220601</v>
@@ -1932,34 +2061,34 @@
         <v>41</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>119</v>
+        <v>123</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>120</v>
+        <v>124</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>119</v>
+        <v>123</v>
       </c>
       <c r="F7" s="2" t="n">
         <v>1</v>
       </c>
       <c r="G7" s="2" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="H7" s="2" t="s">
-        <v>144</v>
+        <v>148</v>
       </c>
       <c r="I7" s="2" t="s">
-        <v>145</v>
+        <v>149</v>
       </c>
       <c r="J7" s="2" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="K7" s="1" t="s">
         <v>43</v>
       </c>
       <c r="L7" s="2" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="M7" s="2" t="n">
         <v>19860101</v>
@@ -1979,34 +2108,34 @@
         <v>47</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>119</v>
+        <v>123</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>120</v>
+        <v>124</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>119</v>
+        <v>123</v>
       </c>
       <c r="F8" s="2" t="n">
         <v>1</v>
       </c>
       <c r="G8" s="2" t="s">
-        <v>146</v>
+        <v>150</v>
       </c>
       <c r="H8" s="2" t="s">
-        <v>147</v>
+        <v>151</v>
       </c>
       <c r="I8" s="2" t="s">
-        <v>148</v>
+        <v>152</v>
       </c>
       <c r="J8" s="2" t="s">
-        <v>149</v>
+        <v>153</v>
       </c>
       <c r="K8" s="1" t="s">
         <v>35</v>
       </c>
       <c r="L8" s="2" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="M8" s="2" t="n">
         <v>20150401</v>

</xml_diff>